<commit_message>
phase B drop the probability tensor from the MXL likelihood
</commit_message>
<xml_diff>
--- a/examples/output/LC_MMNL.xlsx
+++ b/examples/output/LC_MMNL.xlsx
@@ -525,22 +525,22 @@
         <v>8</v>
       </c>
       <c r="B2">
-        <v>-0.0301488924403291</v>
+        <v>-0.030148892440329072</v>
       </c>
       <c r="C2">
         <v>0.05284487336596205</v>
       </c>
       <c r="D2">
-        <v>-0.5705168830955761</v>
+        <v>-0.5705168830955757</v>
       </c>
       <c r="E2">
-        <v>0.5683271744974254</v>
+        <v>0.5683271744974256</v>
       </c>
       <c r="F2">
-        <v>0.058601101043099145</v>
+        <v>0.05860110104309913</v>
       </c>
       <c r="G2">
-        <v>-0.5144765525507038</v>
+        <v>-0.5144765525507035</v>
       </c>
       <c r="H2">
         <v>0.606918849561513</v>
@@ -577,22 +577,22 @@
         <v>10</v>
       </c>
       <c r="B4">
-        <v>-0.7031025794109204</v>
+        <v>-0.7031025794109195</v>
       </c>
       <c r="C4">
-        <v>0.11243415063321031</v>
+        <v>0.1124341506332101</v>
       </c>
       <c r="D4">
-        <v>-6.253461029866498</v>
+        <v>-6.253461029866502</v>
       </c>
       <c r="E4">
         <v>4.014548693476172e-10</v>
       </c>
       <c r="F4">
-        <v>0.23110214866865636</v>
+        <v>0.2311021486686548</v>
       </c>
       <c r="G4">
-        <v>-3.0423887595220784</v>
+        <v>-3.042388759522095</v>
       </c>
       <c r="H4">
         <v>0.002347085507421909</v>
@@ -603,22 +603,22 @@
         <v>11</v>
       </c>
       <c r="B5">
-        <v>-2.9451071726896876</v>
+        <v>-2.9451071726896854</v>
       </c>
       <c r="C5">
-        <v>0.30228874816832424</v>
+        <v>0.30228874816832335</v>
       </c>
       <c r="D5">
-        <v>-9.742695322055969</v>
+        <v>-9.74269532205599</v>
       </c>
       <c r="E5">
         <v>0.0</v>
       </c>
       <c r="F5">
-        <v>0.3474595422256433</v>
+        <v>0.34745954222564224</v>
       </c>
       <c r="G5">
-        <v>-8.47611538835537</v>
+        <v>-8.476115388355389</v>
       </c>
       <c r="H5">
         <v>0.0</v>
@@ -629,25 +629,25 @@
         <v>12</v>
       </c>
       <c r="B6">
-        <v>-0.34005590086442045</v>
+        <v>-0.34005590086442206</v>
       </c>
       <c r="C6">
-        <v>0.27211371042886257</v>
+        <v>0.27211371042886173</v>
       </c>
       <c r="D6">
-        <v>-1.249683084062461</v>
+        <v>-1.2496830840624709</v>
       </c>
       <c r="E6">
-        <v>0.21141533907768717</v>
+        <v>0.21141533907768362</v>
       </c>
       <c r="F6">
-        <v>0.39663183826084736</v>
+        <v>0.39663183826084314</v>
       </c>
       <c r="G6">
-        <v>-0.857359062135553</v>
+        <v>-0.8573590621355662</v>
       </c>
       <c r="H6">
-        <v>0.3912464765809216</v>
+        <v>0.3912464765809145</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -684,22 +684,22 @@
         <v>0.4917618276950913</v>
       </c>
       <c r="C8">
-        <v>0.293570468262593</v>
+        <v>0.2935704682625931</v>
       </c>
       <c r="D8">
-        <v>1.6751065957193627</v>
+        <v>1.675106595719362</v>
       </c>
       <c r="E8">
-        <v>0.09391331909537848</v>
+        <v>0.0939133190953787</v>
       </c>
       <c r="F8">
-        <v>0.33020368910550874</v>
+        <v>0.33020368910550946</v>
       </c>
       <c r="G8">
-        <v>1.489268121223081</v>
+        <v>1.4892681212230776</v>
       </c>
       <c r="H8">
-        <v>0.13641677878843406</v>
+        <v>0.13641677878843494</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -733,25 +733,25 @@
         <v>16</v>
       </c>
       <c r="B10">
-        <v>-0.1102397743707262</v>
+        <v>-0.11023977437072692</v>
       </c>
       <c r="C10">
-        <v>0.3449415894697764</v>
+        <v>0.34494158946977643</v>
       </c>
       <c r="D10">
-        <v>-0.319589686300745</v>
+        <v>-0.319589686300747</v>
       </c>
       <c r="E10">
-        <v>0.7492793938001794</v>
+        <v>0.7492793938001778</v>
       </c>
       <c r="F10">
-        <v>0.39621731459487314</v>
+        <v>0.396217314594873</v>
       </c>
       <c r="G10">
-        <v>-0.27823058283923024</v>
+        <v>-0.27823058283923213</v>
       </c>
       <c r="H10">
-        <v>0.7808353596304205</v>
+        <v>0.780835359630419</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -785,22 +785,22 @@
         <v>18</v>
       </c>
       <c r="B12">
-        <v>-0.042671723765582675</v>
+        <v>-0.042671723765582655</v>
       </c>
       <c r="C12">
-        <v>0.004029968525084044</v>
+        <v>0.004029968525084042</v>
       </c>
       <c r="D12">
-        <v>-10.58859976200255</v>
+        <v>-10.588599762002548</v>
       </c>
       <c r="E12">
         <v>0.0</v>
       </c>
       <c r="F12">
-        <v>0.008256022993292257</v>
+        <v>0.008256022993292226</v>
       </c>
       <c r="G12">
-        <v>-5.168556797897974</v>
+        <v>-5.168556797897991</v>
       </c>
       <c r="H12">
         <v>2.3590859687949717e-7</v>
@@ -811,22 +811,22 @@
         <v>19</v>
       </c>
       <c r="B13">
-        <v>-0.05600992332140068</v>
+        <v>-0.056009923321400736</v>
       </c>
       <c r="C13">
-        <v>0.005594357815475465</v>
+        <v>0.005594357815475466</v>
       </c>
       <c r="D13">
-        <v>-10.011859299822135</v>
+        <v>-10.011859299822143</v>
       </c>
       <c r="E13">
         <v>0.0</v>
       </c>
       <c r="F13">
-        <v>0.008376869585344286</v>
+        <v>0.00837686958534429</v>
       </c>
       <c r="G13">
-        <v>-6.686259437462485</v>
+        <v>-6.686259437462487</v>
       </c>
       <c r="H13">
         <v>2.2894797169215053e-11</v>
@@ -837,22 +837,22 @@
         <v>20</v>
       </c>
       <c r="B14">
-        <v>-3.1343794150488176</v>
+        <v>-3.1343794150488185</v>
       </c>
       <c r="C14">
-        <v>0.2076260764065324</v>
+        <v>0.20762607640653238</v>
       </c>
       <c r="D14">
-        <v>-15.096270513303416</v>
+        <v>-15.096270513303423</v>
       </c>
       <c r="E14">
         <v>0.0</v>
       </c>
       <c r="F14">
-        <v>0.2493185481879971</v>
+        <v>0.2493185481879962</v>
       </c>
       <c r="G14">
-        <v>-12.571785925391152</v>
+        <v>-12.5717859253912</v>
       </c>
       <c r="H14">
         <v>0.0</v>
@@ -866,19 +866,19 @@
         <v>0.7459363064423936</v>
       </c>
       <c r="C15">
-        <v>0.145391622207354</v>
+        <v>0.14539162220735424</v>
       </c>
       <c r="D15">
-        <v>5.130531561017714</v>
+        <v>5.130531561017706</v>
       </c>
       <c r="E15">
         <v>2.8892510917089e-7</v>
       </c>
       <c r="F15">
-        <v>0.13943261379391061</v>
+        <v>0.13943261379391078</v>
       </c>
       <c r="G15">
-        <v>5.349797914173295</v>
+        <v>5.349797914173289</v>
       </c>
       <c r="H15">
         <v>8.805250018006916e-8</v>
@@ -889,22 +889,22 @@
         <v>22</v>
       </c>
       <c r="B16">
-        <v>-1.599195885997084</v>
+        <v>-1.599195885997085</v>
       </c>
       <c r="C16">
-        <v>0.1570622190245036</v>
+        <v>0.1570622190245031</v>
       </c>
       <c r="D16">
-        <v>-10.181925964942533</v>
+        <v>-10.18192596494257</v>
       </c>
       <c r="E16">
         <v>0.0</v>
       </c>
       <c r="F16">
-        <v>0.2317304185228859</v>
+        <v>0.23173041852288345</v>
       </c>
       <c r="G16">
-        <v>-6.901104724148013</v>
+        <v>-6.901104724148089</v>
       </c>
       <c r="H16">
         <v>5.1598725292478775e-12</v>
@@ -915,22 +915,22 @@
         <v>23</v>
       </c>
       <c r="B17">
-        <v>0.5719110365737694</v>
+        <v>0.5719110365737698</v>
       </c>
       <c r="C17">
-        <v>0.09038485542025822</v>
+        <v>0.0903848554202584</v>
       </c>
       <c r="D17">
-        <v>6.327509558040243</v>
+        <v>6.327509558040236</v>
       </c>
       <c r="E17">
         <v>2.491495898482299e-10</v>
       </c>
       <c r="F17">
-        <v>0.10900401167529518</v>
+        <v>0.10900401167529553</v>
       </c>
       <c r="G17">
-        <v>5.246697142462952</v>
+        <v>5.2466971424629385</v>
       </c>
       <c r="H17">
         <v>1.548501371573252e-7</v>
@@ -941,22 +941,22 @@
         <v>24</v>
       </c>
       <c r="B18">
-        <v>-0.0838879871865226</v>
+        <v>-0.08388798718652249</v>
       </c>
       <c r="C18">
-        <v>0.01963738493811367</v>
+        <v>0.01963738493811364</v>
       </c>
       <c r="D18">
-        <v>-4.271851239403403</v>
+        <v>-4.271851239403404</v>
       </c>
       <c r="E18">
         <v>1.9385688656115008e-5</v>
       </c>
       <c r="F18">
-        <v>0.017865635368866813</v>
+        <v>0.017865635368866734</v>
       </c>
       <c r="G18">
-        <v>-4.695494196232635</v>
+        <v>-4.695494196232649</v>
       </c>
       <c r="H18">
         <v>2.6596292013181255e-6</v>
@@ -967,25 +967,25 @@
         <v>25</v>
       </c>
       <c r="B19">
-        <v>-0.818300470638351</v>
+        <v>-0.81830047063835</v>
       </c>
       <c r="C19">
-        <v>0.14139807961006717</v>
+        <v>0.14139807961006629</v>
       </c>
       <c r="D19">
-        <v>-5.787210638892511</v>
+        <v>-5.787210638892541</v>
       </c>
       <c r="E19">
         <v>7.1564816295222045e-9</v>
       </c>
       <c r="F19">
-        <v>0.31783206552488613</v>
+        <v>0.31783206552488213</v>
       </c>
       <c r="G19">
-        <v>-2.5746315724530895</v>
+        <v>-2.574631572453119</v>
       </c>
       <c r="H19">
-        <v>0.010034691245780492</v>
+        <v>0.010034691245779603</v>
       </c>
     </row>
   </sheetData>
@@ -1003,7 +1003,7 @@
         <v>26</v>
       </c>
       <c r="B1">
-        <v>-1497.8720282700492</v>
+        <v>-1497.872028270049</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -1043,7 +1043,7 @@
         <v>32</v>
       </c>
       <c r="B6">
-        <v>175.94235277175903</v>
+        <v>80.9410171508789</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -1067,7 +1067,7 @@
         <v>35</v>
       </c>
       <c r="B9">
-        <v>3023.7440565400984</v>
+        <v>3023.744056540098</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -1075,7 +1075,7 @@
         <v>36</v>
       </c>
       <c r="B10">
-        <v>3109.9592753775314</v>
+        <v>3109.959275377531</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -1083,7 +1083,7 @@
         <v>37</v>
       </c>
       <c r="B11">
-        <v>0.38116479178937057</v>
+        <v>0.3811647917893707</v>
       </c>
     </row>
   </sheetData>

</xml_diff>